<commit_message>
modified init files to add more scenarios
</commit_message>
<xml_diff>
--- a/notebooks/CalSim3DataExtractionInitFile_v4.xlsx
+++ b/notebooks/CalSim3DataExtractionInitFile_v4.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44E45B7B-A643-4B5E-A0CC-5A50D4116B3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8904BB5A-98A0-425C-A3A6-C429F2EB54BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11,6 +11,7 @@
     <sheet name="Init" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -234,25 +235,25 @@
     <t>O475</t>
   </si>
   <si>
-    <t>A36</t>
-  </si>
-  <si>
-    <t>B36</t>
-  </si>
-  <si>
-    <t>C36</t>
-  </si>
-  <si>
-    <t>G36</t>
-  </si>
-  <si>
-    <t>H36</t>
-  </si>
-  <si>
-    <t>I36</t>
-  </si>
-  <si>
-    <t>J36</t>
+    <t>A39</t>
+  </si>
+  <si>
+    <t>B39</t>
+  </si>
+  <si>
+    <t>C39</t>
+  </si>
+  <si>
+    <t>G39</t>
+  </si>
+  <si>
+    <t>H39</t>
+  </si>
+  <si>
+    <t>I39</t>
+  </si>
+  <si>
+    <t>J39</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
added more vaariables to data extraction
</commit_message>
<xml_diff>
--- a/notebooks/CalSim3DataExtractionInitFile_v4.xlsx
+++ b/notebooks/CalSim3DataExtractionInitFile_v4.xlsx
@@ -3,15 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B046A1E-B53D-4330-BC3C-87A7A335F574}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F30EAF47-4D5A-4934-B553-AC074BCB798E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-2700" yWindow="-21720" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Init" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -232,9 +231,6 @@
     <t>O475</t>
   </si>
   <si>
-    <t>E261</t>
-  </si>
-  <si>
     <t>A46</t>
   </si>
   <si>
@@ -254,6 +250,9 @@
   </si>
   <si>
     <t>J46</t>
+  </si>
+  <si>
+    <t>E265</t>
   </si>
 </sst>
 </file>
@@ -647,7 +646,7 @@
         <v>7</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E5" s="2"/>
     </row>
@@ -662,7 +661,7 @@
         <v>35</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E6" s="2"/>
     </row>
@@ -677,7 +676,7 @@
         <v>19</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E7" s="2"/>
     </row>
@@ -692,7 +691,7 @@
         <v>20</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E8" s="2"/>
     </row>
@@ -707,7 +706,7 @@
         <v>21</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E9" s="2"/>
     </row>
@@ -722,7 +721,7 @@
         <v>22</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E10" s="2"/>
     </row>
@@ -737,7 +736,7 @@
         <v>37</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E11" s="2"/>
     </row>
@@ -776,7 +775,7 @@
         <v>25</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
added variable to extraction list
</commit_message>
<xml_diff>
--- a/notebooks/CalSim3DataExtractionInitFile_v4.xlsx
+++ b/notebooks/CalSim3DataExtractionInitFile_v4.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F30EAF47-4D5A-4934-B553-AC074BCB798E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B5D5FF8-7C63-4E0F-9BD9-CF046BC665AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-2700" yWindow="-21720" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Init" sheetId="1" r:id="rId1"/>
@@ -252,7 +252,7 @@
     <t>J46</t>
   </si>
   <si>
-    <t>E265</t>
+    <t>E266</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
added drinking water scenarios
</commit_message>
<xml_diff>
--- a/notebooks/CalSim3DataExtractionInitFile_v4.xlsx
+++ b/notebooks/CalSim3DataExtractionInitFile_v4.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B5D5FF8-7C63-4E0F-9BD9-CF046BC665AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84B4E43D-1504-49A6-9F8E-DB4B60AAC5D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Init" sheetId="1" r:id="rId1"/>
@@ -231,28 +231,28 @@
     <t>O475</t>
   </si>
   <si>
-    <t>A46</t>
-  </si>
-  <si>
-    <t>B46</t>
-  </si>
-  <si>
-    <t>C46</t>
-  </si>
-  <si>
-    <t>G46</t>
-  </si>
-  <si>
-    <t>H46</t>
-  </si>
-  <si>
-    <t>I46</t>
-  </si>
-  <si>
-    <t>J46</t>
-  </si>
-  <si>
     <t>E266</t>
+  </si>
+  <si>
+    <t>A49</t>
+  </si>
+  <si>
+    <t>B49</t>
+  </si>
+  <si>
+    <t>C49</t>
+  </si>
+  <si>
+    <t>G49</t>
+  </si>
+  <si>
+    <t>H49</t>
+  </si>
+  <si>
+    <t>I49</t>
+  </si>
+  <si>
+    <t>J49</t>
   </si>
 </sst>
 </file>
@@ -646,7 +646,7 @@
         <v>7</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E5" s="2"/>
     </row>
@@ -661,7 +661,7 @@
         <v>35</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E6" s="2"/>
     </row>
@@ -676,7 +676,7 @@
         <v>19</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E7" s="2"/>
     </row>
@@ -691,7 +691,7 @@
         <v>20</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E8" s="2"/>
     </row>
@@ -706,7 +706,7 @@
         <v>21</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E9" s="2"/>
     </row>
@@ -721,7 +721,7 @@
         <v>22</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E10" s="2"/>
     </row>
@@ -736,7 +736,7 @@
         <v>37</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E11" s="2"/>
     </row>
@@ -775,7 +775,7 @@
         <v>25</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
trimmed scenarios to historical only
</commit_message>
<xml_diff>
--- a/notebooks/CalSim3DataExtractionInitFile_v4.xlsx
+++ b/notebooks/CalSim3DataExtractionInitFile_v4.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84B4E43D-1504-49A6-9F8E-DB4B60AAC5D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{785AE97A-D20C-4B89-A0C8-ADCD6442E913}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -234,25 +234,25 @@
     <t>E266</t>
   </si>
   <si>
-    <t>A49</t>
-  </si>
-  <si>
-    <t>B49</t>
-  </si>
-  <si>
-    <t>C49</t>
-  </si>
-  <si>
-    <t>G49</t>
-  </si>
-  <si>
-    <t>H49</t>
-  </si>
-  <si>
-    <t>I49</t>
-  </si>
-  <si>
-    <t>J49</t>
+    <t>A25</t>
+  </si>
+  <si>
+    <t>B25</t>
+  </si>
+  <si>
+    <t>C25</t>
+  </si>
+  <si>
+    <t>G25</t>
+  </si>
+  <si>
+    <t>H25</t>
+  </si>
+  <si>
+    <t>I25</t>
+  </si>
+  <si>
+    <t>J25</t>
   </si>
 </sst>
 </file>

</xml_diff>